<commit_message>
Updated Cache with Memory + time limit
</commit_message>
<xml_diff>
--- a/benchmark/new_results/no_cache.xlsx
+++ b/benchmark/new_results/no_cache.xlsx
@@ -518,34 +518,34 @@
         <v>0</v>
       </c>
       <c r="G2" t="n">
-        <v>1000</v>
+        <v>888</v>
       </c>
       <c r="H2" t="n">
         <v>0</v>
       </c>
       <c r="I2" t="n">
-        <v>3.4858</v>
+        <v>5.4805</v>
       </c>
       <c r="J2" t="n">
-        <v>286.88</v>
+        <v>182.47</v>
       </c>
       <c r="K2" t="n">
-        <v>2.1029</v>
+        <v>3.1422</v>
       </c>
       <c r="L2" t="n">
-        <v>2.0133</v>
+        <v>3.0153</v>
       </c>
       <c r="M2" t="n">
-        <v>0.552</v>
+        <v>1.0215</v>
       </c>
       <c r="N2" t="n">
-        <v>3.3347</v>
+        <v>5.2221</v>
       </c>
       <c r="O2" t="n">
-        <v>118.63</v>
+        <v>121.24</v>
       </c>
       <c r="P2" t="n">
-        <v>125.62</v>
+        <v>125.98</v>
       </c>
     </row>
     <row r="3">
@@ -568,34 +568,34 @@
         <v>0</v>
       </c>
       <c r="G3" t="n">
-        <v>1000</v>
+        <v>859</v>
       </c>
       <c r="H3" t="n">
         <v>0</v>
       </c>
       <c r="I3" t="n">
-        <v>3.6901</v>
+        <v>6.49</v>
       </c>
       <c r="J3" t="n">
-        <v>271</v>
+        <v>154.08</v>
       </c>
       <c r="K3" t="n">
-        <v>2.4497</v>
+        <v>4.3747</v>
       </c>
       <c r="L3" t="n">
-        <v>2.1143</v>
+        <v>3.8296</v>
       </c>
       <c r="M3" t="n">
-        <v>0.612</v>
+        <v>0.9595</v>
       </c>
       <c r="N3" t="n">
-        <v>3.3744</v>
+        <v>5.9916</v>
       </c>
       <c r="O3" t="n">
-        <v>141.72</v>
+        <v>146.84</v>
       </c>
       <c r="P3" t="n">
-        <v>152.79</v>
+        <v>153.23</v>
       </c>
     </row>
     <row r="4">
@@ -618,34 +618,34 @@
         <v>0</v>
       </c>
       <c r="G4" t="n">
-        <v>5000</v>
+        <v>4192</v>
       </c>
       <c r="H4" t="n">
         <v>0</v>
       </c>
       <c r="I4" t="n">
-        <v>16.6074</v>
+        <v>29.9696</v>
       </c>
       <c r="J4" t="n">
-        <v>301.07</v>
+        <v>166.84</v>
       </c>
       <c r="K4" t="n">
-        <v>8.749000000000001</v>
+        <v>15.4889</v>
       </c>
       <c r="L4" t="n">
-        <v>8.808299999999999</v>
+        <v>15.5668</v>
       </c>
       <c r="M4" t="n">
-        <v>0.5566</v>
+        <v>1.0785</v>
       </c>
       <c r="N4" t="n">
-        <v>16.1399</v>
+        <v>29.1342</v>
       </c>
       <c r="O4" t="n">
-        <v>158.54</v>
+        <v>159.99</v>
       </c>
       <c r="P4" t="n">
-        <v>161.52</v>
+        <v>161.81</v>
       </c>
     </row>
     <row r="5">
@@ -668,34 +668,34 @@
         <v>0</v>
       </c>
       <c r="G5" t="n">
-        <v>5000</v>
+        <v>4158</v>
       </c>
       <c r="H5" t="n">
         <v>0</v>
       </c>
       <c r="I5" t="n">
-        <v>16.7185</v>
+        <v>29.0236</v>
       </c>
       <c r="J5" t="n">
-        <v>299.07</v>
+        <v>172.27</v>
       </c>
       <c r="K5" t="n">
-        <v>9.141400000000001</v>
+        <v>15.667</v>
       </c>
       <c r="L5" t="n">
-        <v>9.513</v>
+        <v>16.4887</v>
       </c>
       <c r="M5" t="n">
-        <v>0.7211</v>
+        <v>1.1651</v>
       </c>
       <c r="N5" t="n">
-        <v>16.1566</v>
+        <v>28.2157</v>
       </c>
       <c r="O5" t="n">
-        <v>179.6</v>
+        <v>181.15</v>
       </c>
       <c r="P5" t="n">
-        <v>182.66</v>
+        <v>183.12</v>
       </c>
     </row>
     <row r="6">
@@ -718,34 +718,34 @@
         <v>0</v>
       </c>
       <c r="G6" t="n">
-        <v>10000</v>
+        <v>8399</v>
       </c>
       <c r="H6" t="n">
         <v>0</v>
       </c>
       <c r="I6" t="n">
-        <v>36.5167</v>
+        <v>58.5561</v>
       </c>
       <c r="J6" t="n">
-        <v>273.85</v>
+        <v>170.78</v>
       </c>
       <c r="K6" t="n">
-        <v>17.7289</v>
+        <v>29.5934</v>
       </c>
       <c r="L6" t="n">
-        <v>17.5018</v>
+        <v>29.7324</v>
       </c>
       <c r="M6" t="n">
-        <v>0.8676</v>
+        <v>1.5113</v>
       </c>
       <c r="N6" t="n">
-        <v>35.7286</v>
+        <v>57.2184</v>
       </c>
       <c r="O6" t="n">
-        <v>194.81</v>
+        <v>195.95</v>
       </c>
       <c r="P6" t="n">
-        <v>198.7</v>
+        <v>199.7</v>
       </c>
     </row>
     <row r="7">
@@ -768,34 +768,34 @@
         <v>0</v>
       </c>
       <c r="G7" t="n">
-        <v>10000</v>
+        <v>8355</v>
       </c>
       <c r="H7" t="n">
         <v>0</v>
       </c>
       <c r="I7" t="n">
-        <v>51.4159</v>
+        <v>58.7123</v>
       </c>
       <c r="J7" t="n">
-        <v>194.49</v>
+        <v>170.32</v>
       </c>
       <c r="K7" t="n">
-        <v>26.3892</v>
+        <v>30.4653</v>
       </c>
       <c r="L7" t="n">
-        <v>26.3423</v>
+        <v>30.7183</v>
       </c>
       <c r="M7" t="n">
-        <v>1.9073</v>
+        <v>2.1663</v>
       </c>
       <c r="N7" t="n">
-        <v>49.8501</v>
+        <v>57.1722</v>
       </c>
       <c r="O7" t="n">
-        <v>216.64</v>
+        <v>217.5</v>
       </c>
       <c r="P7" t="n">
-        <v>219.73</v>
+        <v>220.23</v>
       </c>
     </row>
     <row r="8">
@@ -809,43 +809,43 @@
         <v>1000</v>
       </c>
       <c r="D8" t="n">
-        <v>848</v>
+        <v>1000</v>
       </c>
       <c r="E8" t="n">
-        <v>152</v>
+        <v>0</v>
       </c>
       <c r="F8" t="n">
         <v>0</v>
       </c>
       <c r="G8" t="n">
-        <v>848</v>
+        <v>938</v>
       </c>
       <c r="H8" t="n">
         <v>0</v>
       </c>
       <c r="I8" t="n">
-        <v>120.5397</v>
+        <v>8.0358</v>
       </c>
       <c r="J8" t="n">
-        <v>7.04</v>
+        <v>124.44</v>
       </c>
       <c r="K8" t="n">
-        <v>1.6063</v>
+        <v>3.7502</v>
       </c>
       <c r="L8" t="n">
-        <v>1.6476</v>
+        <v>3.716</v>
       </c>
       <c r="M8" t="n">
-        <v>0.389</v>
+        <v>0.6345</v>
       </c>
       <c r="N8" t="n">
-        <v>2.8583</v>
+        <v>7.5808</v>
       </c>
       <c r="O8" t="n">
-        <v>171.01</v>
+        <v>176.96</v>
       </c>
       <c r="P8" t="n">
-        <v>178.61</v>
+        <v>179.31</v>
       </c>
     </row>
     <row r="9">
@@ -859,43 +859,43 @@
         <v>1000</v>
       </c>
       <c r="D9" t="n">
-        <v>489</v>
+        <v>693</v>
       </c>
       <c r="E9" t="n">
-        <v>511</v>
+        <v>307</v>
       </c>
       <c r="F9" t="n">
         <v>0</v>
       </c>
       <c r="G9" t="n">
-        <v>489</v>
+        <v>610</v>
       </c>
       <c r="H9" t="n">
         <v>0</v>
       </c>
       <c r="I9" t="n">
-        <v>120.9913</v>
+        <v>121.9287</v>
       </c>
       <c r="J9" t="n">
-        <v>4.04</v>
+        <v>5.68</v>
       </c>
       <c r="K9" t="n">
-        <v>1.3007</v>
+        <v>5.4021</v>
       </c>
       <c r="L9" t="n">
-        <v>1.2951</v>
+        <v>5.76</v>
       </c>
       <c r="M9" t="n">
-        <v>0.5583</v>
+        <v>1.76</v>
       </c>
       <c r="N9" t="n">
-        <v>2.0586</v>
+        <v>6.7254</v>
       </c>
       <c r="O9" t="n">
-        <v>183.89</v>
+        <v>174.67</v>
       </c>
       <c r="P9" t="n">
-        <v>187.84</v>
+        <v>190.61</v>
       </c>
     </row>
     <row r="10">
@@ -918,34 +918,34 @@
         <v>0</v>
       </c>
       <c r="G10" t="n">
-        <v>5000</v>
+        <v>4151</v>
       </c>
       <c r="H10" t="n">
         <v>0</v>
       </c>
       <c r="I10" t="n">
-        <v>27.3387</v>
+        <v>17.0917</v>
       </c>
       <c r="J10" t="n">
-        <v>182.89</v>
+        <v>292.54</v>
       </c>
       <c r="K10" t="n">
-        <v>16.6289</v>
+        <v>8.767099999999999</v>
       </c>
       <c r="L10" t="n">
-        <v>17.28</v>
+        <v>8.595800000000001</v>
       </c>
       <c r="M10" t="n">
-        <v>1.4807</v>
+        <v>0.9751</v>
       </c>
       <c r="N10" t="n">
-        <v>26.1226</v>
+        <v>16.3451</v>
       </c>
       <c r="O10" t="n">
-        <v>170.2</v>
+        <v>170.5</v>
       </c>
       <c r="P10" t="n">
-        <v>171.49</v>
+        <v>173.44</v>
       </c>
     </row>
     <row r="11">
@@ -959,43 +959,43 @@
         <v>5000</v>
       </c>
       <c r="D11" t="n">
-        <v>0</v>
+        <v>5000</v>
       </c>
       <c r="E11" t="n">
-        <v>5000</v>
+        <v>0</v>
       </c>
       <c r="F11" t="n">
         <v>0</v>
       </c>
       <c r="G11" t="n">
-        <v>0</v>
+        <v>4227</v>
       </c>
       <c r="H11" t="n">
         <v>0</v>
       </c>
       <c r="I11" t="n">
-        <v>121.5294</v>
+        <v>15.7464</v>
       </c>
       <c r="J11" t="n">
-        <v>0</v>
+        <v>317.53</v>
       </c>
       <c r="K11" t="n">
-        <v>0</v>
+        <v>8.402900000000001</v>
       </c>
       <c r="L11" t="n">
-        <v>0</v>
+        <v>8.370799999999999</v>
       </c>
       <c r="M11" t="n">
-        <v>0</v>
+        <v>0.8268</v>
       </c>
       <c r="N11" t="n">
-        <v>0</v>
+        <v>15.0042</v>
       </c>
       <c r="O11" t="n">
-        <v>186.91</v>
+        <v>187.75</v>
       </c>
       <c r="P11" t="n">
-        <v>187.53</v>
+        <v>190.43</v>
       </c>
     </row>
     <row r="12">
@@ -1009,43 +1009,43 @@
         <v>10000</v>
       </c>
       <c r="D12" t="n">
-        <v>0</v>
+        <v>10000</v>
       </c>
       <c r="E12" t="n">
-        <v>10000</v>
+        <v>0</v>
       </c>
       <c r="F12" t="n">
         <v>0</v>
       </c>
       <c r="G12" t="n">
-        <v>0</v>
+        <v>8392</v>
       </c>
       <c r="H12" t="n">
         <v>0</v>
       </c>
       <c r="I12" t="n">
-        <v>69.7953</v>
+        <v>30.1026</v>
       </c>
       <c r="J12" t="n">
-        <v>0</v>
+        <v>332.2</v>
       </c>
       <c r="K12" t="n">
-        <v>0</v>
+        <v>15.1512</v>
       </c>
       <c r="L12" t="n">
-        <v>0</v>
+        <v>15.0515</v>
       </c>
       <c r="M12" t="n">
-        <v>0</v>
+        <v>1.4028</v>
       </c>
       <c r="N12" t="n">
-        <v>0</v>
+        <v>28.7389</v>
       </c>
       <c r="O12" t="n">
-        <v>176.29</v>
+        <v>195.86</v>
       </c>
       <c r="P12" t="n">
-        <v>180.2</v>
+        <v>199.71</v>
       </c>
     </row>
     <row r="13">
@@ -1059,43 +1059,43 @@
         <v>10000</v>
       </c>
       <c r="D13" t="n">
-        <v>0</v>
+        <v>10000</v>
       </c>
       <c r="E13" t="n">
-        <v>10000</v>
+        <v>0</v>
       </c>
       <c r="F13" t="n">
         <v>0</v>
       </c>
       <c r="G13" t="n">
-        <v>0</v>
+        <v>8418</v>
       </c>
       <c r="H13" t="n">
         <v>0</v>
       </c>
       <c r="I13" t="n">
-        <v>35.364</v>
+        <v>31.2995</v>
       </c>
       <c r="J13" t="n">
-        <v>0</v>
+        <v>319.49</v>
       </c>
       <c r="K13" t="n">
-        <v>0</v>
+        <v>16.2231</v>
       </c>
       <c r="L13" t="n">
-        <v>0</v>
+        <v>16.2893</v>
       </c>
       <c r="M13" t="n">
-        <v>0</v>
+        <v>1.4909</v>
       </c>
       <c r="N13" t="n">
-        <v>0</v>
+        <v>29.8729</v>
       </c>
       <c r="O13" t="n">
-        <v>178.25</v>
+        <v>217.44</v>
       </c>
       <c r="P13" t="n">
-        <v>181.64</v>
+        <v>220.85</v>
       </c>
     </row>
     <row r="14">
@@ -1109,43 +1109,43 @@
         <v>1000</v>
       </c>
       <c r="D14" t="n">
-        <v>0</v>
+        <v>1000</v>
       </c>
       <c r="E14" t="n">
-        <v>1000</v>
+        <v>0</v>
       </c>
       <c r="F14" t="n">
         <v>0</v>
       </c>
       <c r="G14" t="n">
-        <v>0</v>
+        <v>958</v>
       </c>
       <c r="H14" t="n">
         <v>0</v>
       </c>
       <c r="I14" t="n">
-        <v>8.2568</v>
+        <v>1.9491</v>
       </c>
       <c r="J14" t="n">
-        <v>0</v>
+        <v>513.0599999999999</v>
       </c>
       <c r="K14" t="n">
-        <v>0</v>
+        <v>1.039</v>
       </c>
       <c r="L14" t="n">
-        <v>0</v>
+        <v>1.0215</v>
       </c>
       <c r="M14" t="n">
-        <v>0</v>
+        <v>0.4532</v>
       </c>
       <c r="N14" t="n">
-        <v>0</v>
+        <v>1.6087</v>
       </c>
       <c r="O14" t="n">
-        <v>173.25</v>
+        <v>179.97</v>
       </c>
       <c r="P14" t="n">
-        <v>173.7</v>
+        <v>189.24</v>
       </c>
     </row>
     <row r="15">
@@ -1159,43 +1159,43 @@
         <v>1000</v>
       </c>
       <c r="D15" t="n">
-        <v>0</v>
+        <v>1000</v>
       </c>
       <c r="E15" t="n">
-        <v>1000</v>
+        <v>0</v>
       </c>
       <c r="F15" t="n">
         <v>0</v>
       </c>
       <c r="G15" t="n">
-        <v>0</v>
+        <v>914</v>
       </c>
       <c r="H15" t="n">
         <v>0</v>
       </c>
       <c r="I15" t="n">
-        <v>4.2204</v>
+        <v>2.2423</v>
       </c>
       <c r="J15" t="n">
-        <v>0</v>
+        <v>445.97</v>
       </c>
       <c r="K15" t="n">
-        <v>0</v>
+        <v>1.3166</v>
       </c>
       <c r="L15" t="n">
-        <v>0</v>
+        <v>1.3951</v>
       </c>
       <c r="M15" t="n">
-        <v>0</v>
+        <v>0.7282</v>
       </c>
       <c r="N15" t="n">
-        <v>0</v>
+        <v>1.6573</v>
       </c>
       <c r="O15" t="n">
-        <v>172.87</v>
+        <v>191.33</v>
       </c>
       <c r="P15" t="n">
-        <v>172.89</v>
+        <v>203.82</v>
       </c>
     </row>
     <row r="16">
@@ -1209,43 +1209,43 @@
         <v>5000</v>
       </c>
       <c r="D16" t="n">
-        <v>0</v>
+        <v>5000</v>
       </c>
       <c r="E16" t="n">
-        <v>5000</v>
+        <v>0</v>
       </c>
       <c r="F16" t="n">
         <v>0</v>
       </c>
       <c r="G16" t="n">
-        <v>0</v>
+        <v>4214</v>
       </c>
       <c r="H16" t="n">
         <v>0</v>
       </c>
       <c r="I16" t="n">
-        <v>34.9363</v>
+        <v>7.8605</v>
       </c>
       <c r="J16" t="n">
-        <v>0</v>
+        <v>636.09</v>
       </c>
       <c r="K16" t="n">
-        <v>0</v>
+        <v>3.8995</v>
       </c>
       <c r="L16" t="n">
-        <v>0</v>
+        <v>3.9792</v>
       </c>
       <c r="M16" t="n">
-        <v>0</v>
+        <v>0.5363</v>
       </c>
       <c r="N16" t="n">
-        <v>0</v>
+        <v>7.1668</v>
       </c>
       <c r="O16" t="n">
-        <v>174.95</v>
+        <v>176.39</v>
       </c>
       <c r="P16" t="n">
-        <v>176.14</v>
+        <v>179.25</v>
       </c>
     </row>
     <row r="17">
@@ -1259,43 +1259,43 @@
         <v>5000</v>
       </c>
       <c r="D17" t="n">
-        <v>0</v>
+        <v>5000</v>
       </c>
       <c r="E17" t="n">
-        <v>5000</v>
+        <v>0</v>
       </c>
       <c r="F17" t="n">
         <v>0</v>
       </c>
       <c r="G17" t="n">
-        <v>0</v>
+        <v>4209</v>
       </c>
       <c r="H17" t="n">
         <v>0</v>
       </c>
       <c r="I17" t="n">
-        <v>18.5058</v>
+        <v>8.3911</v>
       </c>
       <c r="J17" t="n">
-        <v>0</v>
+        <v>595.87</v>
       </c>
       <c r="K17" t="n">
-        <v>0</v>
+        <v>4.1424</v>
       </c>
       <c r="L17" t="n">
-        <v>0</v>
+        <v>4.0753</v>
       </c>
       <c r="M17" t="n">
-        <v>0</v>
+        <v>0.8821</v>
       </c>
       <c r="N17" t="n">
-        <v>0</v>
+        <v>7.5429</v>
       </c>
       <c r="O17" t="n">
-        <v>167.56</v>
+        <v>192.71</v>
       </c>
       <c r="P17" t="n">
-        <v>167.93</v>
+        <v>197.49</v>
       </c>
     </row>
     <row r="18">
@@ -1309,43 +1309,43 @@
         <v>10000</v>
       </c>
       <c r="D18" t="n">
-        <v>0</v>
+        <v>10000</v>
       </c>
       <c r="E18" t="n">
-        <v>10000</v>
+        <v>0</v>
       </c>
       <c r="F18" t="n">
         <v>0</v>
       </c>
       <c r="G18" t="n">
-        <v>0</v>
+        <v>8383</v>
       </c>
       <c r="H18" t="n">
         <v>0</v>
       </c>
       <c r="I18" t="n">
-        <v>69.63890000000001</v>
+        <v>34.5595</v>
       </c>
       <c r="J18" t="n">
-        <v>0</v>
+        <v>289.36</v>
       </c>
       <c r="K18" t="n">
-        <v>0</v>
+        <v>19.9066</v>
       </c>
       <c r="L18" t="n">
-        <v>0</v>
+        <v>26.3943</v>
       </c>
       <c r="M18" t="n">
-        <v>0</v>
+        <v>1.307</v>
       </c>
       <c r="N18" t="n">
-        <v>0</v>
+        <v>33.1536</v>
       </c>
       <c r="O18" t="n">
-        <v>177.14</v>
+        <v>197.09</v>
       </c>
       <c r="P18" t="n">
-        <v>179.94</v>
+        <v>199.99</v>
       </c>
     </row>
     <row r="19">
@@ -1359,43 +1359,43 @@
         <v>10000</v>
       </c>
       <c r="D19" t="n">
-        <v>0</v>
+        <v>10000</v>
       </c>
       <c r="E19" t="n">
-        <v>10000</v>
+        <v>0</v>
       </c>
       <c r="F19" t="n">
         <v>0</v>
       </c>
       <c r="G19" t="n">
-        <v>0</v>
+        <v>8352</v>
       </c>
       <c r="H19" t="n">
         <v>0</v>
       </c>
       <c r="I19" t="n">
-        <v>35.1382</v>
+        <v>16.405</v>
       </c>
       <c r="J19" t="n">
-        <v>0</v>
+        <v>609.5700000000001</v>
       </c>
       <c r="K19" t="n">
-        <v>0</v>
+        <v>8.0732</v>
       </c>
       <c r="L19" t="n">
-        <v>0</v>
+        <v>8.146100000000001</v>
       </c>
       <c r="M19" t="n">
-        <v>0</v>
+        <v>1.5351</v>
       </c>
       <c r="N19" t="n">
-        <v>0</v>
+        <v>14.9182</v>
       </c>
       <c r="O19" t="n">
-        <v>178.68</v>
+        <v>215.92</v>
       </c>
       <c r="P19" t="n">
-        <v>181.14</v>
+        <v>220.96</v>
       </c>
     </row>
   </sheetData>

</xml_diff>